<commit_message>
Atualizar lista IO via TIA Openness
</commit_message>
<xml_diff>
--- a/outputs/io-lista/Lista_IO_Editavel_Import_TIA.xlsx
+++ b/outputs/io-lista/Lista_IO_Editavel_Import_TIA.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLC Tags" sheetId="1" r:id="R3d4439f867774bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLC Tags" sheetId="1" r:id="R5653c1ff17b4464c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -74,10 +74,12 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
@@ -303,11 +305,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="13" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="76" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -536,7 +538,7 @@
         <x:v>Entradas_CPU_Local</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>RESERVA_I1_4</x:v>
+        <x:v>STOP_COMP</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>Bool</x:v>
@@ -545,7 +547,7 @@
         <x:v>%I1.4</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>Reserva Tecnica Local CPU</x:v>
+        <x:v>Paragem Local / Botao Cogumelo de Paragem Compactador (Contacto NF)</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -820,7 +822,7 @@
         <x:v>Sensor Optoeletronico de Nivel da Moega a 75%</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="24" hidden="0" customHeight="1">
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="10" t="str">
         <x:v>Entradas_Expansao1_SM1221</x:v>
       </x:c>
@@ -1148,7 +1150,7 @@
         <x:v>Entradas_Expansao3_SM1221</x:v>
       </x:c>
       <x:c r="B50" s="10" t="str">
-        <x:v>RESERVA_I6_2</x:v>
+        <x:v>STOP6_GERAL</x:v>
       </x:c>
       <x:c r="C50" s="10" t="str">
         <x:v>Bool</x:v>
@@ -1157,7 +1159,7 @@
         <x:v>%I6.2</x:v>
       </x:c>
       <x:c r="E50" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DI 3</x:v>
+        <x:v>Paragem Local / Botao Cogumelo de Paragem Geral (Contacto NF)</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -1383,104 +1385,104 @@
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B64" s="10" t="str">
-        <x:v>KM1</x:v>
+        <x:v>OK_SISTEMA</x:v>
       </x:c>
       <x:c r="C64" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D64" s="10" t="str">
-        <x:v>%Q0.0</x:v>
+        <x:v>%M0.0</x:v>
       </x:c>
       <x:c r="E64" s="10" t="str">
-        <x:v>Contactor de Processo do Motor M1 (Tapete 1)</x:v>
+        <x:v>Permissivo geral do sistema (calculado em FC1)</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B65" s="10" t="str">
-        <x:v>KM2</x:v>
+        <x:v>AUT_LINHA_LIGADA</x:v>
       </x:c>
       <x:c r="C65" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D65" s="10" t="str">
-        <x:v>%Q0.1</x:v>
+        <x:v>%M0.1</x:v>
       </x:c>
       <x:c r="E65" s="10" t="str">
-        <x:v>Contactor de Processo do Motor M2 (Tapete 2)</x:v>
+        <x:v>Selo da linha em modo automatico (FC3)</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B66" s="10" t="str">
-        <x:v>KM3</x:v>
+        <x:v>MODO_MANUAL</x:v>
       </x:c>
       <x:c r="C66" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D66" s="10" t="str">
-        <x:v>%Q0.2</x:v>
+        <x:v>%M0.2</x:v>
       </x:c>
       <x:c r="E66" s="10" t="str">
-        <x:v>Contactor de Processo do Motor M3 (Tapete 3)</x:v>
+        <x:v>Modo manual selecionado (FC2)</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B67" s="10" t="str">
-        <x:v>KM4</x:v>
+        <x:v>CICLO_RECUO</x:v>
       </x:c>
       <x:c r="C67" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D67" s="10" t="str">
-        <x:v>%Q0.3</x:v>
+        <x:v>%M0.3</x:v>
       </x:c>
       <x:c r="E67" s="10" t="str">
-        <x:v>Contactor de Processo do Motor M4 (Tapete 4)</x:v>
+        <x:v>Ciclo de recuo do cilindro hidraulico (FC4)</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B68" s="10" t="str">
-        <x:v>KM5</x:v>
+        <x:v>EMERGENCIA</x:v>
       </x:c>
       <x:c r="C68" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D68" s="10" t="str">
-        <x:v>%Q0.4</x:v>
+        <x:v>%M0.4</x:v>
       </x:c>
       <x:c r="E68" s="10" t="str">
-        <x:v>Contactor de Processo do Motor M5 (Tapete 5)</x:v>
+        <x:v>Paragem de emergencia ativa (FC1)</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="10" t="str">
-        <x:v>Saidas_CPU_Local</x:v>
+        <x:v>Marcadores_Internos</x:v>
       </x:c>
       <x:c r="B69" s="10" t="str">
-        <x:v>START_SS_M6</x:v>
+        <x:v>ETAPA_GRAFCET</x:v>
       </x:c>
       <x:c r="C69" s="10" t="str">
-        <x:v>Bool</x:v>
+        <x:v>Word</x:v>
       </x:c>
       <x:c r="D69" s="10" t="str">
-        <x:v>%Q0.5</x:v>
+        <x:v>%MW2</x:v>
       </x:c>
       <x:c r="E69" s="10" t="str">
-        <x:v>Sinal de Habilitacao / Start da Soft Starter (Bomba M6)</x:v>
+        <x:v>Variavel de etapa atual do GRAFCET (FC5_GRAFCET)</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
@@ -1488,16 +1490,16 @@
         <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B70" s="10" t="str">
-        <x:v>Y1_AVANCA</x:v>
+        <x:v>KM1</x:v>
       </x:c>
       <x:c r="C70" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D70" s="10" t="str">
-        <x:v>%Q0.6</x:v>
+        <x:v>%Q0.0</x:v>
       </x:c>
       <x:c r="E70" s="10" t="str">
-        <x:v>Eletrovalvula de Avanco do Cilindro Hidraulico</x:v>
+        <x:v>Contactor de Processo do Motor M1 (Tapete 1)</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
@@ -1505,16 +1507,16 @@
         <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B71" s="10" t="str">
-        <x:v>Y2_RECUA</x:v>
+        <x:v>KM2</x:v>
       </x:c>
       <x:c r="C71" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D71" s="10" t="str">
-        <x:v>%Q0.7</x:v>
+        <x:v>%Q0.1</x:v>
       </x:c>
       <x:c r="E71" s="10" t="str">
-        <x:v>Eletrovalvula de Recuo do Cilindro Hidraulico</x:v>
+        <x:v>Contactor de Processo do Motor M2 (Tapete 2)</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
@@ -1522,16 +1524,16 @@
         <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B72" s="10" t="str">
-        <x:v>H1_VERDE</x:v>
+        <x:v>KM3</x:v>
       </x:c>
       <x:c r="C72" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D72" s="10" t="str">
-        <x:v>%Q1.0</x:v>
+        <x:v>%Q0.2</x:v>
       </x:c>
       <x:c r="E72" s="10" t="str">
-        <x:v>Sinalizador Luminoso Verde: Linha em Funcionamento / Automatico</x:v>
+        <x:v>Contactor de Processo do Motor M3 (Tapete 3)</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
@@ -1539,118 +1541,118 @@
         <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B73" s="10" t="str">
-        <x:v>H2_AMARELO</x:v>
+        <x:v>KM4</x:v>
       </x:c>
       <x:c r="C73" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D73" s="10" t="str">
-        <x:v>%Q1.1</x:v>
+        <x:v>%Q0.3</x:v>
       </x:c>
       <x:c r="E73" s="10" t="str">
-        <x:v>Sinalizador Luminoso Amarelo: Estado de Prontidao / Standby</x:v>
+        <x:v>Contactor de Processo do Motor M4 (Tapete 4)</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
       <x:c r="A74" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B74" s="10" t="str">
-        <x:v>H13_AUTO</x:v>
+        <x:v>KM5</x:v>
       </x:c>
       <x:c r="C74" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D74" s="10" t="str">
-        <x:v>%Q2.0</x:v>
+        <x:v>%Q0.4</x:v>
       </x:c>
       <x:c r="E74" s="10" t="str">
-        <x:v>Sinalizador: Modo AUTOMATICO Selecionado</x:v>
+        <x:v>Contactor de Processo do Motor M5 (Tapete 5)</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
       <x:c r="A75" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B75" s="10" t="str">
-        <x:v>H14_MANUAL</x:v>
+        <x:v>START_SS_M6</x:v>
       </x:c>
       <x:c r="C75" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D75" s="10" t="str">
-        <x:v>%Q2.1</x:v>
+        <x:v>%Q0.5</x:v>
       </x:c>
       <x:c r="E75" s="10" t="str">
-        <x:v>Sinalizador: Modo MANUAL Selecionado</x:v>
+        <x:v>Sinal de Habilitacao / Start da Soft Starter (Bomba M6)</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
       <x:c r="A76" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B76" s="10" t="str">
-        <x:v>H3_AZUL</x:v>
+        <x:v>Y1_AVANCA</x:v>
       </x:c>
       <x:c r="C76" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D76" s="10" t="str">
-        <x:v>%Q2.3</x:v>
+        <x:v>%Q0.6</x:v>
       </x:c>
       <x:c r="E76" s="10" t="str">
-        <x:v>Sinalizador Azul: Nivel da Moega a 75%</x:v>
+        <x:v>Eletrovalvula de Avanco do Cilindro Hidraulico</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
       <x:c r="A77" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B77" s="10" t="str">
-        <x:v>H4_VERMELHO</x:v>
+        <x:v>Y2_RECUA</x:v>
       </x:c>
       <x:c r="C77" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D77" s="10" t="str">
-        <x:v>%Q2.4</x:v>
+        <x:v>%Q0.7</x:v>
       </x:c>
       <x:c r="E77" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Nivel da Moega a 100%</x:v>
+        <x:v>Eletrovalvula de Recuo do Cilindro Hidraulico</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
       <x:c r="A78" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B78" s="10" t="str">
-        <x:v>H5_VERMELHO</x:v>
+        <x:v>H1_VERDE</x:v>
       </x:c>
       <x:c r="C78" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D78" s="10" t="str">
-        <x:v>%Q2.5</x:v>
+        <x:v>%Q1.0</x:v>
       </x:c>
       <x:c r="E78" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria Geral da Linha</x:v>
+        <x:v>Sinalizador Luminoso Verde: Linha em Funcionamento / Automatico</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="10" t="str">
-        <x:v>Saidas_Expansao1_SM1222</x:v>
+        <x:v>Saidas_CPU_Local</x:v>
       </x:c>
       <x:c r="B79" s="10" t="str">
-        <x:v>H6_VERMELHO</x:v>
+        <x:v>H2_AMARELO</x:v>
       </x:c>
       <x:c r="C79" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D79" s="10" t="str">
-        <x:v>%Q2.6</x:v>
+        <x:v>%Q1.1</x:v>
       </x:c>
       <x:c r="E79" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Compactador</x:v>
+        <x:v>Sinalizador Luminoso Amarelo: Estado de Prontidao / Standby</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
@@ -1658,16 +1660,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B80" s="10" t="str">
-        <x:v>H7_VERMELHO</x:v>
+        <x:v>H13_AUTO</x:v>
       </x:c>
       <x:c r="C80" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D80" s="10" t="str">
-        <x:v>%Q2.7</x:v>
+        <x:v>%Q2.0</x:v>
       </x:c>
       <x:c r="E80" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M1</x:v>
+        <x:v>Sinalizador: Modo AUTOMATICO Selecionado</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
@@ -1675,16 +1677,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B81" s="10" t="str">
-        <x:v>H8_VERMELHO</x:v>
+        <x:v>H14_MANUAL</x:v>
       </x:c>
       <x:c r="C81" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D81" s="10" t="str">
-        <x:v>%Q3.0</x:v>
+        <x:v>%Q2.1</x:v>
       </x:c>
       <x:c r="E81" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M2</x:v>
+        <x:v>Sinalizador: Modo MANUAL Selecionado</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
@@ -1692,16 +1694,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B82" s="10" t="str">
-        <x:v>H9_VERMELHO</x:v>
+        <x:v>RESERVA_Q2_2</x:v>
       </x:c>
       <x:c r="C82" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D82" s="10" t="str">
-        <x:v>%Q3.1</x:v>
+        <x:v>%Q2.2</x:v>
       </x:c>
       <x:c r="E82" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M3</x:v>
+        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
@@ -1709,16 +1711,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B83" s="10" t="str">
-        <x:v>H10_VERMELHO</x:v>
+        <x:v>H3_AZUL</x:v>
       </x:c>
       <x:c r="C83" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D83" s="10" t="str">
-        <x:v>%Q3.2</x:v>
+        <x:v>%Q2.3</x:v>
       </x:c>
       <x:c r="E83" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M4</x:v>
+        <x:v>Sinalizador Azul: Nivel da Moega a 75%</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
@@ -1726,16 +1728,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B84" s="10" t="str">
-        <x:v>H11_VERMELHO</x:v>
+        <x:v>H4_VERMELHO</x:v>
       </x:c>
       <x:c r="C84" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D84" s="10" t="str">
-        <x:v>%Q3.3</x:v>
+        <x:v>%Q2.4</x:v>
       </x:c>
       <x:c r="E84" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M5</x:v>
+        <x:v>Sinalizador Vermelho: Nivel da Moega a 100%</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
@@ -1743,16 +1745,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B85" s="10" t="str">
-        <x:v>H12_VERMELHO</x:v>
+        <x:v>H5_VERMELHO</x:v>
       </x:c>
       <x:c r="C85" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D85" s="10" t="str">
-        <x:v>%Q3.4</x:v>
+        <x:v>%Q2.5</x:v>
       </x:c>
       <x:c r="E85" s="10" t="str">
-        <x:v>Sinalizador Vermelho: Paragem / Avaria da Bomba M6</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria Geral da Linha</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
@@ -1760,16 +1762,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B86" s="10" t="str">
-        <x:v>RESERVA_Q2_2</x:v>
+        <x:v>H6_VERMELHO</x:v>
       </x:c>
       <x:c r="C86" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D86" s="10" t="str">
-        <x:v>%Q2.2</x:v>
+        <x:v>%Q2.6</x:v>
       </x:c>
       <x:c r="E86" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Compactador</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
@@ -1777,16 +1779,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B87" s="10" t="str">
-        <x:v>RESERVA_Q3_5</x:v>
+        <x:v>H7_VERMELHO</x:v>
       </x:c>
       <x:c r="C87" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D87" s="10" t="str">
-        <x:v>%Q3.5</x:v>
+        <x:v>%Q2.7</x:v>
       </x:c>
       <x:c r="E87" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M1</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
@@ -1794,16 +1796,16 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B88" s="10" t="str">
-        <x:v>RESERVA_Q3_6</x:v>
+        <x:v>H8_VERMELHO</x:v>
       </x:c>
       <x:c r="C88" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D88" s="10" t="str">
-        <x:v>%Q3.6</x:v>
+        <x:v>%Q3.0</x:v>
       </x:c>
       <x:c r="E88" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M2</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
@@ -1811,124 +1813,124 @@
         <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B89" s="10" t="str">
-        <x:v>RESERVA_Q3_7</x:v>
+        <x:v>H9_VERMELHO</x:v>
       </x:c>
       <x:c r="C89" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D89" s="10" t="str">
-        <x:v>%Q3.7</x:v>
+        <x:v>%Q3.1</x:v>
       </x:c>
       <x:c r="E89" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M3</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
       <x:c r="A90" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B90" s="10" t="str">
-        <x:v>OK_SISTEMA</x:v>
+        <x:v>H10_VERMELHO</x:v>
       </x:c>
       <x:c r="C90" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D90" s="10" t="str">
-        <x:v>%M0.0</x:v>
+        <x:v>%Q3.2</x:v>
       </x:c>
       <x:c r="E90" s="10" t="str">
-        <x:v>Permissivo geral do sistema (calculado em FC1)</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M4</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
       <x:c r="A91" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B91" s="10" t="str">
-        <x:v>AUT_LINHA_LIGADA</x:v>
+        <x:v>H11_VERMELHO</x:v>
       </x:c>
       <x:c r="C91" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D91" s="10" t="str">
-        <x:v>%M0.1</x:v>
+        <x:v>%Q3.3</x:v>
       </x:c>
       <x:c r="E91" s="10" t="str">
-        <x:v>Selo da linha em modo automatico (FC3)</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria do Motor M5</x:v>
       </x:c>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
       <x:c r="A92" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B92" s="10" t="str">
-        <x:v>MODO_MANUAL</x:v>
+        <x:v>H12_VERMELHO</x:v>
       </x:c>
       <x:c r="C92" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D92" s="10" t="str">
-        <x:v>%M0.2</x:v>
+        <x:v>%Q3.4</x:v>
       </x:c>
       <x:c r="E92" s="10" t="str">
-        <x:v>Modo manual selecionado (FC2)</x:v>
+        <x:v>Sinalizador Vermelho: Paragem / Avaria da Bomba M6</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
       <x:c r="A93" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B93" s="10" t="str">
-        <x:v>CICLO_RECUO</x:v>
+        <x:v>RESERVA_Q3_5</x:v>
       </x:c>
       <x:c r="C93" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D93" s="10" t="str">
-        <x:v>%M0.3</x:v>
+        <x:v>%Q3.5</x:v>
       </x:c>
       <x:c r="E93" s="10" t="str">
-        <x:v>Ciclo de recuo do cilindro hidraulico (FC4)</x:v>
+        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
       </x:c>
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
       <x:c r="A94" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B94" s="10" t="str">
-        <x:v>EMERGENCIA</x:v>
+        <x:v>RESERVA_Q3_6</x:v>
       </x:c>
       <x:c r="C94" s="10" t="str">
         <x:v>Bool</x:v>
       </x:c>
       <x:c r="D94" s="10" t="str">
-        <x:v>%M0.4</x:v>
+        <x:v>%Q3.6</x:v>
       </x:c>
       <x:c r="E94" s="10" t="str">
-        <x:v>Paragem de emergencia ativa (FC1)</x:v>
+        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
       </x:c>
     </x:row>
     <x:row r="95" ht="15" hidden="0" customHeight="1">
       <x:c r="A95" s="10" t="str">
-        <x:v>Marcadores_Internos</x:v>
+        <x:v>Saidas_Expansao1_SM1222</x:v>
       </x:c>
       <x:c r="B95" s="10" t="str">
-        <x:v>ETAPA_GRAFCET</x:v>
+        <x:v>RESERVA_Q3_7</x:v>
       </x:c>
       <x:c r="C95" s="10" t="str">
-        <x:v>Word</x:v>
+        <x:v>Bool</x:v>
       </x:c>
       <x:c r="D95" s="10" t="str">
-        <x:v>%MW2</x:v>
+        <x:v>%Q3.7</x:v>
       </x:c>
       <x:c r="E95" s="10" t="str">
-        <x:v>Variavel de etapa atual do GRAFCET (FC5_GRAFCET)</x:v>
+        <x:v>Reserva Tecnica Modulo DQ 1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71daa587455f4d44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde70d3baa3334f2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
alerações,novas networks, ajustei o stop do compactador
</commit_message>
<xml_diff>
--- a/outputs/io-lista/Lista_IO_Editavel_Import_TIA.xlsx
+++ b/outputs/io-lista/Lista_IO_Editavel_Import_TIA.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLC Tags" sheetId="1" r:id="R5653c1ff17b4464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PLC Tags" sheetId="1" r:id="R1cec786b11844dbb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -538,7 +538,7 @@
         <x:v>Entradas_CPU_Local</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>STOP_COMP</x:v>
+        <x:v>RESERVA_I1_4</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>Bool</x:v>
@@ -547,7 +547,7 @@
         <x:v>%I1.4</x:v>
       </x:c>
       <x:c r="E14" s="10" t="str">
-        <x:v>Paragem Local / Botao Cogumelo de Paragem Compactador (Contacto NF)</x:v>
+        <x:v>Reserva Tecnica Local CPU</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1167,7 +1167,7 @@
         <x:v>Entradas_Expansao3_SM1221</x:v>
       </x:c>
       <x:c r="B51" s="10" t="str">
-        <x:v>RESERVA_I6_3</x:v>
+        <x:v>NA_STOP_COMP</x:v>
       </x:c>
       <x:c r="C51" s="10" t="str">
         <x:v>Bool</x:v>
@@ -1176,7 +1176,7 @@
         <x:v>%I6.3</x:v>
       </x:c>
       <x:c r="E51" s="10" t="str">
-        <x:v>Reserva Tecnica Modulo DI 3</x:v>
+        <x:v>Botao / Paragem Local de Seguranca do Compactador</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
@@ -1930,7 +1930,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde70d3baa3334f2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48a2a57fb8db4a01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>